<commit_message>
fix(assets): the template learns how parcels really group, and the ZIP stays text far down
Vlad's word from the backend: one parcel carries one recipient name, so
gifts merge only on a full recipient-plus-address match; the same door
under different names ships separately. Step one of the instructions
said otherwise and now tells the truth. The ZIP column keeps its text
format to row 500, so a long list pasted past the styled area does not
lose its leading zeros to Excel.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/gildedbox-gifts-template.xlsx
+++ b/assets/gildedbox-gifts-template.xlsx
@@ -152,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -191,6 +191,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -629,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1188,6 +1189,1416 @@
       <c r="K30" s="11" t="n"/>
       <c r="L30" s="11" t="n"/>
       <c r="M30" s="13" t="n"/>
+    </row>
+    <row r="31">
+      <c r="F31" s="14" t="n"/>
+    </row>
+    <row r="32">
+      <c r="F32" s="14" t="n"/>
+    </row>
+    <row r="33">
+      <c r="F33" s="14" t="n"/>
+    </row>
+    <row r="34">
+      <c r="F34" s="14" t="n"/>
+    </row>
+    <row r="35">
+      <c r="F35" s="14" t="n"/>
+    </row>
+    <row r="36">
+      <c r="F36" s="14" t="n"/>
+    </row>
+    <row r="37">
+      <c r="F37" s="14" t="n"/>
+    </row>
+    <row r="38">
+      <c r="F38" s="14" t="n"/>
+    </row>
+    <row r="39">
+      <c r="F39" s="14" t="n"/>
+    </row>
+    <row r="40">
+      <c r="F40" s="14" t="n"/>
+    </row>
+    <row r="41">
+      <c r="F41" s="14" t="n"/>
+    </row>
+    <row r="42">
+      <c r="F42" s="14" t="n"/>
+    </row>
+    <row r="43">
+      <c r="F43" s="14" t="n"/>
+    </row>
+    <row r="44">
+      <c r="F44" s="14" t="n"/>
+    </row>
+    <row r="45">
+      <c r="F45" s="14" t="n"/>
+    </row>
+    <row r="46">
+      <c r="F46" s="14" t="n"/>
+    </row>
+    <row r="47">
+      <c r="F47" s="14" t="n"/>
+    </row>
+    <row r="48">
+      <c r="F48" s="14" t="n"/>
+    </row>
+    <row r="49">
+      <c r="F49" s="14" t="n"/>
+    </row>
+    <row r="50">
+      <c r="F50" s="14" t="n"/>
+    </row>
+    <row r="51">
+      <c r="F51" s="14" t="n"/>
+    </row>
+    <row r="52">
+      <c r="F52" s="14" t="n"/>
+    </row>
+    <row r="53">
+      <c r="F53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="F54" s="14" t="n"/>
+    </row>
+    <row r="55">
+      <c r="F55" s="14" t="n"/>
+    </row>
+    <row r="56">
+      <c r="F56" s="14" t="n"/>
+    </row>
+    <row r="57">
+      <c r="F57" s="14" t="n"/>
+    </row>
+    <row r="58">
+      <c r="F58" s="14" t="n"/>
+    </row>
+    <row r="59">
+      <c r="F59" s="14" t="n"/>
+    </row>
+    <row r="60">
+      <c r="F60" s="14" t="n"/>
+    </row>
+    <row r="61">
+      <c r="F61" s="14" t="n"/>
+    </row>
+    <row r="62">
+      <c r="F62" s="14" t="n"/>
+    </row>
+    <row r="63">
+      <c r="F63" s="14" t="n"/>
+    </row>
+    <row r="64">
+      <c r="F64" s="14" t="n"/>
+    </row>
+    <row r="65">
+      <c r="F65" s="14" t="n"/>
+    </row>
+    <row r="66">
+      <c r="F66" s="14" t="n"/>
+    </row>
+    <row r="67">
+      <c r="F67" s="14" t="n"/>
+    </row>
+    <row r="68">
+      <c r="F68" s="14" t="n"/>
+    </row>
+    <row r="69">
+      <c r="F69" s="14" t="n"/>
+    </row>
+    <row r="70">
+      <c r="F70" s="14" t="n"/>
+    </row>
+    <row r="71">
+      <c r="F71" s="14" t="n"/>
+    </row>
+    <row r="72">
+      <c r="F72" s="14" t="n"/>
+    </row>
+    <row r="73">
+      <c r="F73" s="14" t="n"/>
+    </row>
+    <row r="74">
+      <c r="F74" s="14" t="n"/>
+    </row>
+    <row r="75">
+      <c r="F75" s="14" t="n"/>
+    </row>
+    <row r="76">
+      <c r="F76" s="14" t="n"/>
+    </row>
+    <row r="77">
+      <c r="F77" s="14" t="n"/>
+    </row>
+    <row r="78">
+      <c r="F78" s="14" t="n"/>
+    </row>
+    <row r="79">
+      <c r="F79" s="14" t="n"/>
+    </row>
+    <row r="80">
+      <c r="F80" s="14" t="n"/>
+    </row>
+    <row r="81">
+      <c r="F81" s="14" t="n"/>
+    </row>
+    <row r="82">
+      <c r="F82" s="14" t="n"/>
+    </row>
+    <row r="83">
+      <c r="F83" s="14" t="n"/>
+    </row>
+    <row r="84">
+      <c r="F84" s="14" t="n"/>
+    </row>
+    <row r="85">
+      <c r="F85" s="14" t="n"/>
+    </row>
+    <row r="86">
+      <c r="F86" s="14" t="n"/>
+    </row>
+    <row r="87">
+      <c r="F87" s="14" t="n"/>
+    </row>
+    <row r="88">
+      <c r="F88" s="14" t="n"/>
+    </row>
+    <row r="89">
+      <c r="F89" s="14" t="n"/>
+    </row>
+    <row r="90">
+      <c r="F90" s="14" t="n"/>
+    </row>
+    <row r="91">
+      <c r="F91" s="14" t="n"/>
+    </row>
+    <row r="92">
+      <c r="F92" s="14" t="n"/>
+    </row>
+    <row r="93">
+      <c r="F93" s="14" t="n"/>
+    </row>
+    <row r="94">
+      <c r="F94" s="14" t="n"/>
+    </row>
+    <row r="95">
+      <c r="F95" s="14" t="n"/>
+    </row>
+    <row r="96">
+      <c r="F96" s="14" t="n"/>
+    </row>
+    <row r="97">
+      <c r="F97" s="14" t="n"/>
+    </row>
+    <row r="98">
+      <c r="F98" s="14" t="n"/>
+    </row>
+    <row r="99">
+      <c r="F99" s="14" t="n"/>
+    </row>
+    <row r="100">
+      <c r="F100" s="14" t="n"/>
+    </row>
+    <row r="101">
+      <c r="F101" s="14" t="n"/>
+    </row>
+    <row r="102">
+      <c r="F102" s="14" t="n"/>
+    </row>
+    <row r="103">
+      <c r="F103" s="14" t="n"/>
+    </row>
+    <row r="104">
+      <c r="F104" s="14" t="n"/>
+    </row>
+    <row r="105">
+      <c r="F105" s="14" t="n"/>
+    </row>
+    <row r="106">
+      <c r="F106" s="14" t="n"/>
+    </row>
+    <row r="107">
+      <c r="F107" s="14" t="n"/>
+    </row>
+    <row r="108">
+      <c r="F108" s="14" t="n"/>
+    </row>
+    <row r="109">
+      <c r="F109" s="14" t="n"/>
+    </row>
+    <row r="110">
+      <c r="F110" s="14" t="n"/>
+    </row>
+    <row r="111">
+      <c r="F111" s="14" t="n"/>
+    </row>
+    <row r="112">
+      <c r="F112" s="14" t="n"/>
+    </row>
+    <row r="113">
+      <c r="F113" s="14" t="n"/>
+    </row>
+    <row r="114">
+      <c r="F114" s="14" t="n"/>
+    </row>
+    <row r="115">
+      <c r="F115" s="14" t="n"/>
+    </row>
+    <row r="116">
+      <c r="F116" s="14" t="n"/>
+    </row>
+    <row r="117">
+      <c r="F117" s="14" t="n"/>
+    </row>
+    <row r="118">
+      <c r="F118" s="14" t="n"/>
+    </row>
+    <row r="119">
+      <c r="F119" s="14" t="n"/>
+    </row>
+    <row r="120">
+      <c r="F120" s="14" t="n"/>
+    </row>
+    <row r="121">
+      <c r="F121" s="14" t="n"/>
+    </row>
+    <row r="122">
+      <c r="F122" s="14" t="n"/>
+    </row>
+    <row r="123">
+      <c r="F123" s="14" t="n"/>
+    </row>
+    <row r="124">
+      <c r="F124" s="14" t="n"/>
+    </row>
+    <row r="125">
+      <c r="F125" s="14" t="n"/>
+    </row>
+    <row r="126">
+      <c r="F126" s="14" t="n"/>
+    </row>
+    <row r="127">
+      <c r="F127" s="14" t="n"/>
+    </row>
+    <row r="128">
+      <c r="F128" s="14" t="n"/>
+    </row>
+    <row r="129">
+      <c r="F129" s="14" t="n"/>
+    </row>
+    <row r="130">
+      <c r="F130" s="14" t="n"/>
+    </row>
+    <row r="131">
+      <c r="F131" s="14" t="n"/>
+    </row>
+    <row r="132">
+      <c r="F132" s="14" t="n"/>
+    </row>
+    <row r="133">
+      <c r="F133" s="14" t="n"/>
+    </row>
+    <row r="134">
+      <c r="F134" s="14" t="n"/>
+    </row>
+    <row r="135">
+      <c r="F135" s="14" t="n"/>
+    </row>
+    <row r="136">
+      <c r="F136" s="14" t="n"/>
+    </row>
+    <row r="137">
+      <c r="F137" s="14" t="n"/>
+    </row>
+    <row r="138">
+      <c r="F138" s="14" t="n"/>
+    </row>
+    <row r="139">
+      <c r="F139" s="14" t="n"/>
+    </row>
+    <row r="140">
+      <c r="F140" s="14" t="n"/>
+    </row>
+    <row r="141">
+      <c r="F141" s="14" t="n"/>
+    </row>
+    <row r="142">
+      <c r="F142" s="14" t="n"/>
+    </row>
+    <row r="143">
+      <c r="F143" s="14" t="n"/>
+    </row>
+    <row r="144">
+      <c r="F144" s="14" t="n"/>
+    </row>
+    <row r="145">
+      <c r="F145" s="14" t="n"/>
+    </row>
+    <row r="146">
+      <c r="F146" s="14" t="n"/>
+    </row>
+    <row r="147">
+      <c r="F147" s="14" t="n"/>
+    </row>
+    <row r="148">
+      <c r="F148" s="14" t="n"/>
+    </row>
+    <row r="149">
+      <c r="F149" s="14" t="n"/>
+    </row>
+    <row r="150">
+      <c r="F150" s="14" t="n"/>
+    </row>
+    <row r="151">
+      <c r="F151" s="14" t="n"/>
+    </row>
+    <row r="152">
+      <c r="F152" s="14" t="n"/>
+    </row>
+    <row r="153">
+      <c r="F153" s="14" t="n"/>
+    </row>
+    <row r="154">
+      <c r="F154" s="14" t="n"/>
+    </row>
+    <row r="155">
+      <c r="F155" s="14" t="n"/>
+    </row>
+    <row r="156">
+      <c r="F156" s="14" t="n"/>
+    </row>
+    <row r="157">
+      <c r="F157" s="14" t="n"/>
+    </row>
+    <row r="158">
+      <c r="F158" s="14" t="n"/>
+    </row>
+    <row r="159">
+      <c r="F159" s="14" t="n"/>
+    </row>
+    <row r="160">
+      <c r="F160" s="14" t="n"/>
+    </row>
+    <row r="161">
+      <c r="F161" s="14" t="n"/>
+    </row>
+    <row r="162">
+      <c r="F162" s="14" t="n"/>
+    </row>
+    <row r="163">
+      <c r="F163" s="14" t="n"/>
+    </row>
+    <row r="164">
+      <c r="F164" s="14" t="n"/>
+    </row>
+    <row r="165">
+      <c r="F165" s="14" t="n"/>
+    </row>
+    <row r="166">
+      <c r="F166" s="14" t="n"/>
+    </row>
+    <row r="167">
+      <c r="F167" s="14" t="n"/>
+    </row>
+    <row r="168">
+      <c r="F168" s="14" t="n"/>
+    </row>
+    <row r="169">
+      <c r="F169" s="14" t="n"/>
+    </row>
+    <row r="170">
+      <c r="F170" s="14" t="n"/>
+    </row>
+    <row r="171">
+      <c r="F171" s="14" t="n"/>
+    </row>
+    <row r="172">
+      <c r="F172" s="14" t="n"/>
+    </row>
+    <row r="173">
+      <c r="F173" s="14" t="n"/>
+    </row>
+    <row r="174">
+      <c r="F174" s="14" t="n"/>
+    </row>
+    <row r="175">
+      <c r="F175" s="14" t="n"/>
+    </row>
+    <row r="176">
+      <c r="F176" s="14" t="n"/>
+    </row>
+    <row r="177">
+      <c r="F177" s="14" t="n"/>
+    </row>
+    <row r="178">
+      <c r="F178" s="14" t="n"/>
+    </row>
+    <row r="179">
+      <c r="F179" s="14" t="n"/>
+    </row>
+    <row r="180">
+      <c r="F180" s="14" t="n"/>
+    </row>
+    <row r="181">
+      <c r="F181" s="14" t="n"/>
+    </row>
+    <row r="182">
+      <c r="F182" s="14" t="n"/>
+    </row>
+    <row r="183">
+      <c r="F183" s="14" t="n"/>
+    </row>
+    <row r="184">
+      <c r="F184" s="14" t="n"/>
+    </row>
+    <row r="185">
+      <c r="F185" s="14" t="n"/>
+    </row>
+    <row r="186">
+      <c r="F186" s="14" t="n"/>
+    </row>
+    <row r="187">
+      <c r="F187" s="14" t="n"/>
+    </row>
+    <row r="188">
+      <c r="F188" s="14" t="n"/>
+    </row>
+    <row r="189">
+      <c r="F189" s="14" t="n"/>
+    </row>
+    <row r="190">
+      <c r="F190" s="14" t="n"/>
+    </row>
+    <row r="191">
+      <c r="F191" s="14" t="n"/>
+    </row>
+    <row r="192">
+      <c r="F192" s="14" t="n"/>
+    </row>
+    <row r="193">
+      <c r="F193" s="14" t="n"/>
+    </row>
+    <row r="194">
+      <c r="F194" s="14" t="n"/>
+    </row>
+    <row r="195">
+      <c r="F195" s="14" t="n"/>
+    </row>
+    <row r="196">
+      <c r="F196" s="14" t="n"/>
+    </row>
+    <row r="197">
+      <c r="F197" s="14" t="n"/>
+    </row>
+    <row r="198">
+      <c r="F198" s="14" t="n"/>
+    </row>
+    <row r="199">
+      <c r="F199" s="14" t="n"/>
+    </row>
+    <row r="200">
+      <c r="F200" s="14" t="n"/>
+    </row>
+    <row r="201">
+      <c r="F201" s="14" t="n"/>
+    </row>
+    <row r="202">
+      <c r="F202" s="14" t="n"/>
+    </row>
+    <row r="203">
+      <c r="F203" s="14" t="n"/>
+    </row>
+    <row r="204">
+      <c r="F204" s="14" t="n"/>
+    </row>
+    <row r="205">
+      <c r="F205" s="14" t="n"/>
+    </row>
+    <row r="206">
+      <c r="F206" s="14" t="n"/>
+    </row>
+    <row r="207">
+      <c r="F207" s="14" t="n"/>
+    </row>
+    <row r="208">
+      <c r="F208" s="14" t="n"/>
+    </row>
+    <row r="209">
+      <c r="F209" s="14" t="n"/>
+    </row>
+    <row r="210">
+      <c r="F210" s="14" t="n"/>
+    </row>
+    <row r="211">
+      <c r="F211" s="14" t="n"/>
+    </row>
+    <row r="212">
+      <c r="F212" s="14" t="n"/>
+    </row>
+    <row r="213">
+      <c r="F213" s="14" t="n"/>
+    </row>
+    <row r="214">
+      <c r="F214" s="14" t="n"/>
+    </row>
+    <row r="215">
+      <c r="F215" s="14" t="n"/>
+    </row>
+    <row r="216">
+      <c r="F216" s="14" t="n"/>
+    </row>
+    <row r="217">
+      <c r="F217" s="14" t="n"/>
+    </row>
+    <row r="218">
+      <c r="F218" s="14" t="n"/>
+    </row>
+    <row r="219">
+      <c r="F219" s="14" t="n"/>
+    </row>
+    <row r="220">
+      <c r="F220" s="14" t="n"/>
+    </row>
+    <row r="221">
+      <c r="F221" s="14" t="n"/>
+    </row>
+    <row r="222">
+      <c r="F222" s="14" t="n"/>
+    </row>
+    <row r="223">
+      <c r="F223" s="14" t="n"/>
+    </row>
+    <row r="224">
+      <c r="F224" s="14" t="n"/>
+    </row>
+    <row r="225">
+      <c r="F225" s="14" t="n"/>
+    </row>
+    <row r="226">
+      <c r="F226" s="14" t="n"/>
+    </row>
+    <row r="227">
+      <c r="F227" s="14" t="n"/>
+    </row>
+    <row r="228">
+      <c r="F228" s="14" t="n"/>
+    </row>
+    <row r="229">
+      <c r="F229" s="14" t="n"/>
+    </row>
+    <row r="230">
+      <c r="F230" s="14" t="n"/>
+    </row>
+    <row r="231">
+      <c r="F231" s="14" t="n"/>
+    </row>
+    <row r="232">
+      <c r="F232" s="14" t="n"/>
+    </row>
+    <row r="233">
+      <c r="F233" s="14" t="n"/>
+    </row>
+    <row r="234">
+      <c r="F234" s="14" t="n"/>
+    </row>
+    <row r="235">
+      <c r="F235" s="14" t="n"/>
+    </row>
+    <row r="236">
+      <c r="F236" s="14" t="n"/>
+    </row>
+    <row r="237">
+      <c r="F237" s="14" t="n"/>
+    </row>
+    <row r="238">
+      <c r="F238" s="14" t="n"/>
+    </row>
+    <row r="239">
+      <c r="F239" s="14" t="n"/>
+    </row>
+    <row r="240">
+      <c r="F240" s="14" t="n"/>
+    </row>
+    <row r="241">
+      <c r="F241" s="14" t="n"/>
+    </row>
+    <row r="242">
+      <c r="F242" s="14" t="n"/>
+    </row>
+    <row r="243">
+      <c r="F243" s="14" t="n"/>
+    </row>
+    <row r="244">
+      <c r="F244" s="14" t="n"/>
+    </row>
+    <row r="245">
+      <c r="F245" s="14" t="n"/>
+    </row>
+    <row r="246">
+      <c r="F246" s="14" t="n"/>
+    </row>
+    <row r="247">
+      <c r="F247" s="14" t="n"/>
+    </row>
+    <row r="248">
+      <c r="F248" s="14" t="n"/>
+    </row>
+    <row r="249">
+      <c r="F249" s="14" t="n"/>
+    </row>
+    <row r="250">
+      <c r="F250" s="14" t="n"/>
+    </row>
+    <row r="251">
+      <c r="F251" s="14" t="n"/>
+    </row>
+    <row r="252">
+      <c r="F252" s="14" t="n"/>
+    </row>
+    <row r="253">
+      <c r="F253" s="14" t="n"/>
+    </row>
+    <row r="254">
+      <c r="F254" s="14" t="n"/>
+    </row>
+    <row r="255">
+      <c r="F255" s="14" t="n"/>
+    </row>
+    <row r="256">
+      <c r="F256" s="14" t="n"/>
+    </row>
+    <row r="257">
+      <c r="F257" s="14" t="n"/>
+    </row>
+    <row r="258">
+      <c r="F258" s="14" t="n"/>
+    </row>
+    <row r="259">
+      <c r="F259" s="14" t="n"/>
+    </row>
+    <row r="260">
+      <c r="F260" s="14" t="n"/>
+    </row>
+    <row r="261">
+      <c r="F261" s="14" t="n"/>
+    </row>
+    <row r="262">
+      <c r="F262" s="14" t="n"/>
+    </row>
+    <row r="263">
+      <c r="F263" s="14" t="n"/>
+    </row>
+    <row r="264">
+      <c r="F264" s="14" t="n"/>
+    </row>
+    <row r="265">
+      <c r="F265" s="14" t="n"/>
+    </row>
+    <row r="266">
+      <c r="F266" s="14" t="n"/>
+    </row>
+    <row r="267">
+      <c r="F267" s="14" t="n"/>
+    </row>
+    <row r="268">
+      <c r="F268" s="14" t="n"/>
+    </row>
+    <row r="269">
+      <c r="F269" s="14" t="n"/>
+    </row>
+    <row r="270">
+      <c r="F270" s="14" t="n"/>
+    </row>
+    <row r="271">
+      <c r="F271" s="14" t="n"/>
+    </row>
+    <row r="272">
+      <c r="F272" s="14" t="n"/>
+    </row>
+    <row r="273">
+      <c r="F273" s="14" t="n"/>
+    </row>
+    <row r="274">
+      <c r="F274" s="14" t="n"/>
+    </row>
+    <row r="275">
+      <c r="F275" s="14" t="n"/>
+    </row>
+    <row r="276">
+      <c r="F276" s="14" t="n"/>
+    </row>
+    <row r="277">
+      <c r="F277" s="14" t="n"/>
+    </row>
+    <row r="278">
+      <c r="F278" s="14" t="n"/>
+    </row>
+    <row r="279">
+      <c r="F279" s="14" t="n"/>
+    </row>
+    <row r="280">
+      <c r="F280" s="14" t="n"/>
+    </row>
+    <row r="281">
+      <c r="F281" s="14" t="n"/>
+    </row>
+    <row r="282">
+      <c r="F282" s="14" t="n"/>
+    </row>
+    <row r="283">
+      <c r="F283" s="14" t="n"/>
+    </row>
+    <row r="284">
+      <c r="F284" s="14" t="n"/>
+    </row>
+    <row r="285">
+      <c r="F285" s="14" t="n"/>
+    </row>
+    <row r="286">
+      <c r="F286" s="14" t="n"/>
+    </row>
+    <row r="287">
+      <c r="F287" s="14" t="n"/>
+    </row>
+    <row r="288">
+      <c r="F288" s="14" t="n"/>
+    </row>
+    <row r="289">
+      <c r="F289" s="14" t="n"/>
+    </row>
+    <row r="290">
+      <c r="F290" s="14" t="n"/>
+    </row>
+    <row r="291">
+      <c r="F291" s="14" t="n"/>
+    </row>
+    <row r="292">
+      <c r="F292" s="14" t="n"/>
+    </row>
+    <row r="293">
+      <c r="F293" s="14" t="n"/>
+    </row>
+    <row r="294">
+      <c r="F294" s="14" t="n"/>
+    </row>
+    <row r="295">
+      <c r="F295" s="14" t="n"/>
+    </row>
+    <row r="296">
+      <c r="F296" s="14" t="n"/>
+    </row>
+    <row r="297">
+      <c r="F297" s="14" t="n"/>
+    </row>
+    <row r="298">
+      <c r="F298" s="14" t="n"/>
+    </row>
+    <row r="299">
+      <c r="F299" s="14" t="n"/>
+    </row>
+    <row r="300">
+      <c r="F300" s="14" t="n"/>
+    </row>
+    <row r="301">
+      <c r="F301" s="14" t="n"/>
+    </row>
+    <row r="302">
+      <c r="F302" s="14" t="n"/>
+    </row>
+    <row r="303">
+      <c r="F303" s="14" t="n"/>
+    </row>
+    <row r="304">
+      <c r="F304" s="14" t="n"/>
+    </row>
+    <row r="305">
+      <c r="F305" s="14" t="n"/>
+    </row>
+    <row r="306">
+      <c r="F306" s="14" t="n"/>
+    </row>
+    <row r="307">
+      <c r="F307" s="14" t="n"/>
+    </row>
+    <row r="308">
+      <c r="F308" s="14" t="n"/>
+    </row>
+    <row r="309">
+      <c r="F309" s="14" t="n"/>
+    </row>
+    <row r="310">
+      <c r="F310" s="14" t="n"/>
+    </row>
+    <row r="311">
+      <c r="F311" s="14" t="n"/>
+    </row>
+    <row r="312">
+      <c r="F312" s="14" t="n"/>
+    </row>
+    <row r="313">
+      <c r="F313" s="14" t="n"/>
+    </row>
+    <row r="314">
+      <c r="F314" s="14" t="n"/>
+    </row>
+    <row r="315">
+      <c r="F315" s="14" t="n"/>
+    </row>
+    <row r="316">
+      <c r="F316" s="14" t="n"/>
+    </row>
+    <row r="317">
+      <c r="F317" s="14" t="n"/>
+    </row>
+    <row r="318">
+      <c r="F318" s="14" t="n"/>
+    </row>
+    <row r="319">
+      <c r="F319" s="14" t="n"/>
+    </row>
+    <row r="320">
+      <c r="F320" s="14" t="n"/>
+    </row>
+    <row r="321">
+      <c r="F321" s="14" t="n"/>
+    </row>
+    <row r="322">
+      <c r="F322" s="14" t="n"/>
+    </row>
+    <row r="323">
+      <c r="F323" s="14" t="n"/>
+    </row>
+    <row r="324">
+      <c r="F324" s="14" t="n"/>
+    </row>
+    <row r="325">
+      <c r="F325" s="14" t="n"/>
+    </row>
+    <row r="326">
+      <c r="F326" s="14" t="n"/>
+    </row>
+    <row r="327">
+      <c r="F327" s="14" t="n"/>
+    </row>
+    <row r="328">
+      <c r="F328" s="14" t="n"/>
+    </row>
+    <row r="329">
+      <c r="F329" s="14" t="n"/>
+    </row>
+    <row r="330">
+      <c r="F330" s="14" t="n"/>
+    </row>
+    <row r="331">
+      <c r="F331" s="14" t="n"/>
+    </row>
+    <row r="332">
+      <c r="F332" s="14" t="n"/>
+    </row>
+    <row r="333">
+      <c r="F333" s="14" t="n"/>
+    </row>
+    <row r="334">
+      <c r="F334" s="14" t="n"/>
+    </row>
+    <row r="335">
+      <c r="F335" s="14" t="n"/>
+    </row>
+    <row r="336">
+      <c r="F336" s="14" t="n"/>
+    </row>
+    <row r="337">
+      <c r="F337" s="14" t="n"/>
+    </row>
+    <row r="338">
+      <c r="F338" s="14" t="n"/>
+    </row>
+    <row r="339">
+      <c r="F339" s="14" t="n"/>
+    </row>
+    <row r="340">
+      <c r="F340" s="14" t="n"/>
+    </row>
+    <row r="341">
+      <c r="F341" s="14" t="n"/>
+    </row>
+    <row r="342">
+      <c r="F342" s="14" t="n"/>
+    </row>
+    <row r="343">
+      <c r="F343" s="14" t="n"/>
+    </row>
+    <row r="344">
+      <c r="F344" s="14" t="n"/>
+    </row>
+    <row r="345">
+      <c r="F345" s="14" t="n"/>
+    </row>
+    <row r="346">
+      <c r="F346" s="14" t="n"/>
+    </row>
+    <row r="347">
+      <c r="F347" s="14" t="n"/>
+    </row>
+    <row r="348">
+      <c r="F348" s="14" t="n"/>
+    </row>
+    <row r="349">
+      <c r="F349" s="14" t="n"/>
+    </row>
+    <row r="350">
+      <c r="F350" s="14" t="n"/>
+    </row>
+    <row r="351">
+      <c r="F351" s="14" t="n"/>
+    </row>
+    <row r="352">
+      <c r="F352" s="14" t="n"/>
+    </row>
+    <row r="353">
+      <c r="F353" s="14" t="n"/>
+    </row>
+    <row r="354">
+      <c r="F354" s="14" t="n"/>
+    </row>
+    <row r="355">
+      <c r="F355" s="14" t="n"/>
+    </row>
+    <row r="356">
+      <c r="F356" s="14" t="n"/>
+    </row>
+    <row r="357">
+      <c r="F357" s="14" t="n"/>
+    </row>
+    <row r="358">
+      <c r="F358" s="14" t="n"/>
+    </row>
+    <row r="359">
+      <c r="F359" s="14" t="n"/>
+    </row>
+    <row r="360">
+      <c r="F360" s="14" t="n"/>
+    </row>
+    <row r="361">
+      <c r="F361" s="14" t="n"/>
+    </row>
+    <row r="362">
+      <c r="F362" s="14" t="n"/>
+    </row>
+    <row r="363">
+      <c r="F363" s="14" t="n"/>
+    </row>
+    <row r="364">
+      <c r="F364" s="14" t="n"/>
+    </row>
+    <row r="365">
+      <c r="F365" s="14" t="n"/>
+    </row>
+    <row r="366">
+      <c r="F366" s="14" t="n"/>
+    </row>
+    <row r="367">
+      <c r="F367" s="14" t="n"/>
+    </row>
+    <row r="368">
+      <c r="F368" s="14" t="n"/>
+    </row>
+    <row r="369">
+      <c r="F369" s="14" t="n"/>
+    </row>
+    <row r="370">
+      <c r="F370" s="14" t="n"/>
+    </row>
+    <row r="371">
+      <c r="F371" s="14" t="n"/>
+    </row>
+    <row r="372">
+      <c r="F372" s="14" t="n"/>
+    </row>
+    <row r="373">
+      <c r="F373" s="14" t="n"/>
+    </row>
+    <row r="374">
+      <c r="F374" s="14" t="n"/>
+    </row>
+    <row r="375">
+      <c r="F375" s="14" t="n"/>
+    </row>
+    <row r="376">
+      <c r="F376" s="14" t="n"/>
+    </row>
+    <row r="377">
+      <c r="F377" s="14" t="n"/>
+    </row>
+    <row r="378">
+      <c r="F378" s="14" t="n"/>
+    </row>
+    <row r="379">
+      <c r="F379" s="14" t="n"/>
+    </row>
+    <row r="380">
+      <c r="F380" s="14" t="n"/>
+    </row>
+    <row r="381">
+      <c r="F381" s="14" t="n"/>
+    </row>
+    <row r="382">
+      <c r="F382" s="14" t="n"/>
+    </row>
+    <row r="383">
+      <c r="F383" s="14" t="n"/>
+    </row>
+    <row r="384">
+      <c r="F384" s="14" t="n"/>
+    </row>
+    <row r="385">
+      <c r="F385" s="14" t="n"/>
+    </row>
+    <row r="386">
+      <c r="F386" s="14" t="n"/>
+    </row>
+    <row r="387">
+      <c r="F387" s="14" t="n"/>
+    </row>
+    <row r="388">
+      <c r="F388" s="14" t="n"/>
+    </row>
+    <row r="389">
+      <c r="F389" s="14" t="n"/>
+    </row>
+    <row r="390">
+      <c r="F390" s="14" t="n"/>
+    </row>
+    <row r="391">
+      <c r="F391" s="14" t="n"/>
+    </row>
+    <row r="392">
+      <c r="F392" s="14" t="n"/>
+    </row>
+    <row r="393">
+      <c r="F393" s="14" t="n"/>
+    </row>
+    <row r="394">
+      <c r="F394" s="14" t="n"/>
+    </row>
+    <row r="395">
+      <c r="F395" s="14" t="n"/>
+    </row>
+    <row r="396">
+      <c r="F396" s="14" t="n"/>
+    </row>
+    <row r="397">
+      <c r="F397" s="14" t="n"/>
+    </row>
+    <row r="398">
+      <c r="F398" s="14" t="n"/>
+    </row>
+    <row r="399">
+      <c r="F399" s="14" t="n"/>
+    </row>
+    <row r="400">
+      <c r="F400" s="14" t="n"/>
+    </row>
+    <row r="401">
+      <c r="F401" s="14" t="n"/>
+    </row>
+    <row r="402">
+      <c r="F402" s="14" t="n"/>
+    </row>
+    <row r="403">
+      <c r="F403" s="14" t="n"/>
+    </row>
+    <row r="404">
+      <c r="F404" s="14" t="n"/>
+    </row>
+    <row r="405">
+      <c r="F405" s="14" t="n"/>
+    </row>
+    <row r="406">
+      <c r="F406" s="14" t="n"/>
+    </row>
+    <row r="407">
+      <c r="F407" s="14" t="n"/>
+    </row>
+    <row r="408">
+      <c r="F408" s="14" t="n"/>
+    </row>
+    <row r="409">
+      <c r="F409" s="14" t="n"/>
+    </row>
+    <row r="410">
+      <c r="F410" s="14" t="n"/>
+    </row>
+    <row r="411">
+      <c r="F411" s="14" t="n"/>
+    </row>
+    <row r="412">
+      <c r="F412" s="14" t="n"/>
+    </row>
+    <row r="413">
+      <c r="F413" s="14" t="n"/>
+    </row>
+    <row r="414">
+      <c r="F414" s="14" t="n"/>
+    </row>
+    <row r="415">
+      <c r="F415" s="14" t="n"/>
+    </row>
+    <row r="416">
+      <c r="F416" s="14" t="n"/>
+    </row>
+    <row r="417">
+      <c r="F417" s="14" t="n"/>
+    </row>
+    <row r="418">
+      <c r="F418" s="14" t="n"/>
+    </row>
+    <row r="419">
+      <c r="F419" s="14" t="n"/>
+    </row>
+    <row r="420">
+      <c r="F420" s="14" t="n"/>
+    </row>
+    <row r="421">
+      <c r="F421" s="14" t="n"/>
+    </row>
+    <row r="422">
+      <c r="F422" s="14" t="n"/>
+    </row>
+    <row r="423">
+      <c r="F423" s="14" t="n"/>
+    </row>
+    <row r="424">
+      <c r="F424" s="14" t="n"/>
+    </row>
+    <row r="425">
+      <c r="F425" s="14" t="n"/>
+    </row>
+    <row r="426">
+      <c r="F426" s="14" t="n"/>
+    </row>
+    <row r="427">
+      <c r="F427" s="14" t="n"/>
+    </row>
+    <row r="428">
+      <c r="F428" s="14" t="n"/>
+    </row>
+    <row r="429">
+      <c r="F429" s="14" t="n"/>
+    </row>
+    <row r="430">
+      <c r="F430" s="14" t="n"/>
+    </row>
+    <row r="431">
+      <c r="F431" s="14" t="n"/>
+    </row>
+    <row r="432">
+      <c r="F432" s="14" t="n"/>
+    </row>
+    <row r="433">
+      <c r="F433" s="14" t="n"/>
+    </row>
+    <row r="434">
+      <c r="F434" s="14" t="n"/>
+    </row>
+    <row r="435">
+      <c r="F435" s="14" t="n"/>
+    </row>
+    <row r="436">
+      <c r="F436" s="14" t="n"/>
+    </row>
+    <row r="437">
+      <c r="F437" s="14" t="n"/>
+    </row>
+    <row r="438">
+      <c r="F438" s="14" t="n"/>
+    </row>
+    <row r="439">
+      <c r="F439" s="14" t="n"/>
+    </row>
+    <row r="440">
+      <c r="F440" s="14" t="n"/>
+    </row>
+    <row r="441">
+      <c r="F441" s="14" t="n"/>
+    </row>
+    <row r="442">
+      <c r="F442" s="14" t="n"/>
+    </row>
+    <row r="443">
+      <c r="F443" s="14" t="n"/>
+    </row>
+    <row r="444">
+      <c r="F444" s="14" t="n"/>
+    </row>
+    <row r="445">
+      <c r="F445" s="14" t="n"/>
+    </row>
+    <row r="446">
+      <c r="F446" s="14" t="n"/>
+    </row>
+    <row r="447">
+      <c r="F447" s="14" t="n"/>
+    </row>
+    <row r="448">
+      <c r="F448" s="14" t="n"/>
+    </row>
+    <row r="449">
+      <c r="F449" s="14" t="n"/>
+    </row>
+    <row r="450">
+      <c r="F450" s="14" t="n"/>
+    </row>
+    <row r="451">
+      <c r="F451" s="14" t="n"/>
+    </row>
+    <row r="452">
+      <c r="F452" s="14" t="n"/>
+    </row>
+    <row r="453">
+      <c r="F453" s="14" t="n"/>
+    </row>
+    <row r="454">
+      <c r="F454" s="14" t="n"/>
+    </row>
+    <row r="455">
+      <c r="F455" s="14" t="n"/>
+    </row>
+    <row r="456">
+      <c r="F456" s="14" t="n"/>
+    </row>
+    <row r="457">
+      <c r="F457" s="14" t="n"/>
+    </row>
+    <row r="458">
+      <c r="F458" s="14" t="n"/>
+    </row>
+    <row r="459">
+      <c r="F459" s="14" t="n"/>
+    </row>
+    <row r="460">
+      <c r="F460" s="14" t="n"/>
+    </row>
+    <row r="461">
+      <c r="F461" s="14" t="n"/>
+    </row>
+    <row r="462">
+      <c r="F462" s="14" t="n"/>
+    </row>
+    <row r="463">
+      <c r="F463" s="14" t="n"/>
+    </row>
+    <row r="464">
+      <c r="F464" s="14" t="n"/>
+    </row>
+    <row r="465">
+      <c r="F465" s="14" t="n"/>
+    </row>
+    <row r="466">
+      <c r="F466" s="14" t="n"/>
+    </row>
+    <row r="467">
+      <c r="F467" s="14" t="n"/>
+    </row>
+    <row r="468">
+      <c r="F468" s="14" t="n"/>
+    </row>
+    <row r="469">
+      <c r="F469" s="14" t="n"/>
+    </row>
+    <row r="470">
+      <c r="F470" s="14" t="n"/>
+    </row>
+    <row r="471">
+      <c r="F471" s="14" t="n"/>
+    </row>
+    <row r="472">
+      <c r="F472" s="14" t="n"/>
+    </row>
+    <row r="473">
+      <c r="F473" s="14" t="n"/>
+    </row>
+    <row r="474">
+      <c r="F474" s="14" t="n"/>
+    </row>
+    <row r="475">
+      <c r="F475" s="14" t="n"/>
+    </row>
+    <row r="476">
+      <c r="F476" s="14" t="n"/>
+    </row>
+    <row r="477">
+      <c r="F477" s="14" t="n"/>
+    </row>
+    <row r="478">
+      <c r="F478" s="14" t="n"/>
+    </row>
+    <row r="479">
+      <c r="F479" s="14" t="n"/>
+    </row>
+    <row r="480">
+      <c r="F480" s="14" t="n"/>
+    </row>
+    <row r="481">
+      <c r="F481" s="14" t="n"/>
+    </row>
+    <row r="482">
+      <c r="F482" s="14" t="n"/>
+    </row>
+    <row r="483">
+      <c r="F483" s="14" t="n"/>
+    </row>
+    <row r="484">
+      <c r="F484" s="14" t="n"/>
+    </row>
+    <row r="485">
+      <c r="F485" s="14" t="n"/>
+    </row>
+    <row r="486">
+      <c r="F486" s="14" t="n"/>
+    </row>
+    <row r="487">
+      <c r="F487" s="14" t="n"/>
+    </row>
+    <row r="488">
+      <c r="F488" s="14" t="n"/>
+    </row>
+    <row r="489">
+      <c r="F489" s="14" t="n"/>
+    </row>
+    <row r="490">
+      <c r="F490" s="14" t="n"/>
+    </row>
+    <row r="491">
+      <c r="F491" s="14" t="n"/>
+    </row>
+    <row r="492">
+      <c r="F492" s="14" t="n"/>
+    </row>
+    <row r="493">
+      <c r="F493" s="14" t="n"/>
+    </row>
+    <row r="494">
+      <c r="F494" s="14" t="n"/>
+    </row>
+    <row r="495">
+      <c r="F495" s="14" t="n"/>
+    </row>
+    <row r="496">
+      <c r="F496" s="14" t="n"/>
+    </row>
+    <row r="497">
+      <c r="F497" s="14" t="n"/>
+    </row>
+    <row r="498">
+      <c r="F498" s="14" t="n"/>
+    </row>
+    <row r="499">
+      <c r="F499" s="14" t="n"/>
+    </row>
+    <row r="500">
+      <c r="F500" s="14" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1215,147 +2626,147 @@
   </cols>
   <sheetData>
     <row r="2" ht="26" customHeight="1">
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>How to fill this file</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>Five minutes, one pass. Save it when you are done and upload it back in checkout.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>1 · One row is one gift.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Twenty gifts means twenty rows. Rows with the same delivery address ship together, and shipping is charged once per address.</t>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Twenty gifts means twenty rows. Gifts for the same recipient at the same address ship together in one parcel; the same address under different names ships as separate parcels, since every parcel carries one recipient name.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>2 · Delivery columns are required.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Recipient name, Address line 1, City, State, ZIP and Country must be filled on every row. Apt / Suite only when there is one. Type ZIP as text so a leading zero is kept.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>3 · Personalization is optional. All of it.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>A blank cell simply means that part stays unpersonalized; the gift still ships. No need to write N/A or 'blank'.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>4 · Gift reference name is never printed.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>It is your own label for telling gifts apart in a batch (it also helps our graphics team match gifts to people). Recipients never see it.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>5 · Mind the limits.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>Apple AirTag takes up to 3 characters (A–Z, 0–9). Luggage Tag, Passport sleeve and the Presentation box lid take up to 24 characters each.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>6 · Card message.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>One message per gift. Want the same card in every box? Write it once and copy it down the column.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>7 · Upload and check.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>Back in checkout, upload the file. We show every row we read and highlight anything that needs a fix before you continue.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="18" t="inlineStr">
+      <c r="B27" s="19" t="inlineStr">
         <is>
           <t>Three rows, three scenarios</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>· Full personalization: fill every personalization cell (see the gray example row on the Gifts sheet).</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>· Card only: fill Card message, leave the item cells blank.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="B30" s="17" t="inlineStr">
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>· Nothing personal: leave all personalization cells blank. Delivery columns are still required.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="19" t="inlineStr">
+      <c r="B32" s="20" t="inlineStr">
         <is>
           <t>Prefer a plain CSV? Download the CSV template instead: same columns, no styling.</t>
         </is>

</xml_diff>